<commit_message>
Chore: update public excel import template with exact columns matching mockup
</commit_message>
<xml_diff>
--- a/public/template-impor-penerjemah.xlsx
+++ b/public/template-impor-penerjemah.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Template" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,23 +397,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:H2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>No Anggota</v>
+        <v>no_anggota</v>
       </c>
       <c r="B1" t="str">
-        <v>Nama Penerjemah</v>
+        <v>nama_penerjemah</v>
       </c>
       <c r="C1" t="str">
-        <v>Email</v>
+        <v>no_sk_kemenkum</v>
       </c>
       <c r="D1" t="str">
-        <v>SK Kemenkumham</v>
+        <v>tgl_sk</v>
       </c>
       <c r="E1" t="str">
-        <v>Arah Bahasa</v>
+        <v>arah_bahasa</v>
+      </c>
+      <c r="F1" t="str">
+        <v>masa_aktif</v>
+      </c>
+      <c r="G1" t="str">
+        <v>url_foto</v>
+      </c>
+      <c r="H1" t="str">
+        <v>sk_lengkap</v>
       </c>
     </row>
     <row r="2">
@@ -424,35 +433,27 @@
         <v>Muhammad Arifin</v>
       </c>
       <c r="C2" t="str">
-        <v>arifin@example.com</v>
+        <v>AHU-55 AH.03.07.2022</v>
       </c>
       <c r="D2" t="str">
-        <v>AHU-55 AH.03.07.2022 Tanggal 5 Oktober 2022</v>
+        <v>5 Oktober 2022</v>
       </c>
       <c r="E2" t="str">
         <v>Indonesia - Inggris, Inggris - Indonesia, Indonesia - Belanda, Belanda - Indonesia</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>25005</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Zaki Syah Iqbal</v>
-      </c>
-      <c r="C3" t="str">
-        <v>zaki@example.com</v>
-      </c>
-      <c r="D3" t="str">
-        <v>AHU-12 AH.04.01.2023 Tanggal 12 Januari 2023</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Inggris - Indonesia, Indonesia - Inggris</v>
+      <c r="F2" t="str">
+        <v>Seumur Hidup</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>AHU-55 AH.03.07.2022 Tanggal 5 Oktober 2022</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>